<commit_message>
Quartz sync: May 27, 2025, 10:08 PM
</commit_message>
<xml_diff>
--- a/content/Obsidian Functional Stuff/z-All pdfs, Images & Excalidraw Drawing and SVGs/New Microsoft Excel Worksheet.xlsx
+++ b/content/Obsidian Functional Stuff/z-All pdfs, Images & Excalidraw Drawing and SVGs/New Microsoft Excel Worksheet.xlsx
@@ -1,26 +1,70 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chakr\my-notes\content\Obsidian Functional Stuff\z-All pdfs, Images &amp; Excalidraw Drawing and SVGs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA2B03B1-B60C-456F-A797-9FE89DEB8DA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>PV</t>
+  </si>
+  <si>
+    <t>FV</t>
+  </si>
+  <si>
+    <t>t</t>
+  </si>
+  <si>
+    <t>r</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="167" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -46,14 +90,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -330,10 +378,43 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="E3:H4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="8" max="8" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>0</v>
+      </c>
+      <c r="G3" t="s">
+        <v>2</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E4">
+        <v>90000</v>
+      </c>
+      <c r="F4">
+        <v>50000</v>
+      </c>
+      <c r="G4">
+        <v>3</v>
+      </c>
+      <c r="H4" s="2">
+        <f>(((E4/F4)^(1/G4))-1)</f>
+        <v>0.21644039911467994</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>